<commit_message>
GV edit changes only a few validation in edit to be taken care like Finance Month closed and Intsrument date validation in respect to current document date
</commit_message>
<xml_diff>
--- a/src/test/resources/Finance/GeneralVoucher.xlsx
+++ b/src/test/resources/Finance/GeneralVoucher.xlsx
@@ -4,12 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView/>
+    <workbookView windowWidth="20490" windowHeight="6900" firstSheet="4" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="DocumentInformation" sheetId="3" r:id="rId1"/>
     <sheet name="ExpenseIncomeDetail" sheetId="2" r:id="rId2"/>
     <sheet name="SiteAllocation" sheetId="1" r:id="rId3"/>
+    <sheet name="RevertVoucherInfo" sheetId="4" r:id="rId4"/>
+    <sheet name="EditVoucherInfo" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="77">
   <si>
     <t>TestCaseID</t>
   </si>
@@ -130,6 +132,15 @@
     <t>TYPE3</t>
   </si>
   <si>
+    <t>GV-EDIT-002</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Advance tax adjustment (before edit)</t>
+  </si>
+  <si>
     <t>Site Name</t>
   </si>
   <si>
@@ -140,6 +151,117 @@
   </si>
   <si>
     <t>HAPPY SPROUTS-KP Road</t>
+  </si>
+  <si>
+    <t>Existing Voucher No.</t>
+  </si>
+  <si>
+    <t>Release Status</t>
+  </si>
+  <si>
+    <t>FIN-GV-REVERT-01</t>
+  </si>
+  <si>
+    <t>VG/00303/26-27</t>
+  </si>
+  <si>
+    <t>P</t>
+  </si>
+  <si>
+    <t>FIN-GV-REVERT-02</t>
+  </si>
+  <si>
+    <t>VG/00101/26-27</t>
+  </si>
+  <si>
+    <t>FIN-GV-REVERT-03</t>
+  </si>
+  <si>
+    <t>VG/00096/26-27</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
+    <t>Edit Scenario</t>
+  </si>
+  <si>
+    <t>New Reference</t>
+  </si>
+  <si>
+    <t>New Remarks</t>
+  </si>
+  <si>
+    <t>New Date</t>
+  </si>
+  <si>
+    <t>Edited Line No.</t>
+  </si>
+  <si>
+    <t>New Amount</t>
+  </si>
+  <si>
+    <t>New Is Reversal</t>
+  </si>
+  <si>
+    <t>GV-EDIT-001</t>
+  </si>
+  <si>
+    <t>VG/00375/26-27</t>
+  </si>
+  <si>
+    <t>HEADER_ONLY</t>
+  </si>
+  <si>
+    <t>REF-EDIT-01</t>
+  </si>
+  <si>
+    <t>Updated narration for header edit</t>
+  </si>
+  <si>
+    <t>VG/00377/26-27</t>
+  </si>
+  <si>
+    <t>DETAIL_LINE</t>
+  </si>
+  <si>
+    <t>REF-EDIT-02</t>
+  </si>
+  <si>
+    <t>Updated narration for detail edit</t>
+  </si>
+  <si>
+    <t>Entry Method</t>
+  </si>
+  <si>
+    <t>ACTIONS_EDIT</t>
+  </si>
+  <si>
+    <t>GV-EDIT-003</t>
+  </si>
+  <si>
+    <t>VG/00378/26-27</t>
+  </si>
+  <si>
+    <t>REF-EDIT-03</t>
+  </si>
+  <si>
+    <t>Updated narration for header edit (double-click entry)</t>
+  </si>
+  <si>
+    <t>DOUBLE_CLICK_EDIT</t>
+  </si>
+  <si>
+    <t>GV-EDIT-004</t>
+  </si>
+  <si>
+    <t>VG/00379/26-27</t>
+  </si>
+  <si>
+    <t>REF-EDIT-04</t>
+  </si>
+  <si>
+    <t>Updated narration for detail edit (double-click entry)</t>
   </si>
 </sst>
 </file>
@@ -152,13 +274,19 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF333333"/>
+      <name val="Segoe UI"/>
+      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -625,138 +753,144 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
@@ -1290,7 +1424,7 @@
   <dimension ref="A1:F2"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="5"/>
   <cols>
-    <col min="3" max="3" width="9.14285714285714" style="1"/>
+    <col min="3" max="3" style="3" width="9.14285714285714" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1300,7 +1434,7 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
       <c r="D1" t="s">
@@ -1317,7 +1451,7 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="E2" t="s">
@@ -1336,17 +1470,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3"/>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4"/>
   <cols>
-    <col min="2" max="2" width="9.14285714285714" style="1"/>
+    <col min="1" max="1" customWidth="true" width="12.7142857142857" collapsed="true"/>
+    <col min="2" max="2" style="3" width="9.14285714285714" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" width="17.8571428571429" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C1" t="s">
@@ -1378,7 +1514,7 @@
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>19</v>
       </c>
       <c r="C2" t="s">
@@ -1401,7 +1537,7 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C3" t="s">
@@ -1424,7 +1560,7 @@
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C4" t="s">
@@ -1444,6 +1580,38 @@
       </c>
       <c r="J4" t="s">
         <v>32</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F5" t="s">
+        <v>35</v>
+      </c>
+      <c r="G5" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5">
+        <v>900</v>
+      </c>
+      <c r="I5" t="s">
+        <v>34</v>
+      </c>
+      <c r="J5" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1458,32 +1626,32 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="3"/>
   <cols>
-    <col min="2" max="2" width="9.14285714285714" style="1"/>
+    <col min="2" max="2" style="3" width="9.14285714285714" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>10</v>
       </c>
       <c r="C1" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="D2">
         <v>900</v>
@@ -1493,11 +1661,11 @@
       <c r="A3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="3" t="s">
         <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D3">
         <v>800</v>
@@ -1507,4 +1675,173 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="2"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="18.8571428571429" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" width="21.1428571428571" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" width="15.0" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelRow="2"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="12.4190476190476" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" width="19.5047619047619" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" width="13.9904761904762" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" width="14.352380952381" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" width="14.7142857142857" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" width="31.5619047619048" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" width="9.85714285714286" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" width="14.5714285714286" collapsed="true"/>
+    <col min="9" max="9" customWidth="true" width="12.8666666666667" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" width="15.0952380952381" collapsed="true"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="J2" t="s" s="0">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="H3" t="n" s="0">
+        <v>1500.0</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="J3" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>